<commit_message>
Manual terminal run — Youth & Tutoring 2026-10-06-0617
</commit_message>
<xml_diff>
--- a/results/auto_Cape_Town_Youth_and_Tutoring.xlsx
+++ b/results/auto_Cape_Town_Youth_and_Tutoring.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="31">
   <si>
     <t>Organisation Name</t>
   </si>
@@ -37,9 +37,6 @@
     <t>Sent</t>
   </si>
   <si>
-    <t>The Shine Centre</t>
-  </si>
-  <si>
     <t>Christel House South Africa</t>
   </si>
   <si>
@@ -67,15 +64,15 @@
     <t>Shine Literacy</t>
   </si>
   <si>
+    <t>Wordworks</t>
+  </si>
+  <si>
     <t>Youth &amp; Tutoring</t>
   </si>
   <si>
     <t>Cape Town</t>
   </si>
   <si>
-    <t>info@shinecentre.org.za</t>
-  </si>
-  <si>
     <t>info@christelhouse.org.za</t>
   </si>
   <si>
@@ -101,6 +98,15 @@
   </si>
   <si>
     <t>info@shineliteracy.org.za</t>
+  </si>
+  <si>
+    <t>info@wordworks.org.za</t>
+  </si>
+  <si>
+    <t>www.wordworks.org.za</t>
+  </si>
+  <si>
+    <t>Yes</t>
   </si>
 </sst>
 </file>
@@ -471,6 +477,9 @@
       <c r="D2" t="s">
         <v>19</v>
       </c>
+      <c r="G2" t="s">
+        <v>30</v>
+      </c>
     </row>
     <row r="3" spans="1:7">
       <c r="A3" t="s">
@@ -485,6 +494,9 @@
       <c r="D3" t="s">
         <v>20</v>
       </c>
+      <c r="G3" t="s">
+        <v>30</v>
+      </c>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" t="s">
@@ -499,6 +511,9 @@
       <c r="D4" t="s">
         <v>21</v>
       </c>
+      <c r="G4" t="s">
+        <v>30</v>
+      </c>
     </row>
     <row r="5" spans="1:7">
       <c r="A5" t="s">
@@ -513,6 +528,9 @@
       <c r="D5" t="s">
         <v>22</v>
       </c>
+      <c r="G5" t="s">
+        <v>30</v>
+      </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" t="s">
@@ -527,6 +545,9 @@
       <c r="D6" t="s">
         <v>23</v>
       </c>
+      <c r="G6" t="s">
+        <v>30</v>
+      </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" t="s">
@@ -541,6 +562,9 @@
       <c r="D7" t="s">
         <v>24</v>
       </c>
+      <c r="G7" t="s">
+        <v>30</v>
+      </c>
     </row>
     <row r="8" spans="1:7">
       <c r="A8" t="s">
@@ -555,6 +579,9 @@
       <c r="D8" t="s">
         <v>25</v>
       </c>
+      <c r="G8" t="s">
+        <v>30</v>
+      </c>
     </row>
     <row r="9" spans="1:7">
       <c r="A9" t="s">
@@ -569,6 +596,9 @@
       <c r="D9" t="s">
         <v>26</v>
       </c>
+      <c r="G9" t="s">
+        <v>30</v>
+      </c>
     </row>
     <row r="10" spans="1:7">
       <c r="A10" t="s">
@@ -583,6 +613,9 @@
       <c r="D10" t="s">
         <v>27</v>
       </c>
+      <c r="G10" t="s">
+        <v>30</v>
+      </c>
     </row>
     <row r="11" spans="1:7">
       <c r="A11" t="s">
@@ -596,6 +629,12 @@
       </c>
       <c r="D11" t="s">
         <v>28</v>
+      </c>
+      <c r="F11" t="s">
+        <v>29</v>
+      </c>
+      <c r="G11" t="s">
+        <v>30</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Manual Youth & Tutoring send 2026-10-06-0716
</commit_message>
<xml_diff>
--- a/results/auto_Cape_Town_Youth_and_Tutoring.xlsx
+++ b/results/auto_Cape_Town_Youth_and_Tutoring.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="61">
   <si>
     <t>Organisation Name</t>
   </si>
@@ -37,73 +37,163 @@
     <t>Sent</t>
   </si>
   <si>
-    <t>Christel House South Africa</t>
-  </si>
-  <si>
-    <t>Bottomup</t>
-  </si>
-  <si>
-    <t>Salesian Life Choices</t>
-  </si>
-  <si>
-    <t>Ikamva Labantu Youth</t>
-  </si>
-  <si>
-    <t>Action Volunteers Africa</t>
-  </si>
-  <si>
-    <t>The President's Award for Youth Empowerment WC</t>
-  </si>
-  <si>
-    <t>Rlabs</t>
-  </si>
-  <si>
-    <t>Ampath Foundation</t>
-  </si>
-  <si>
-    <t>Shine Literacy</t>
-  </si>
-  <si>
-    <t>Wordworks</t>
+    <t>Randburg Youth Centre</t>
+  </si>
+  <si>
+    <t>Randburg Youth Development Programme</t>
+  </si>
+  <si>
+    <t>Randburg Educational Support Services</t>
+  </si>
+  <si>
+    <t>Randburg Youth Empowerment Trust</t>
+  </si>
+  <si>
+    <t>Randburg After‑School Academy</t>
+  </si>
+  <si>
+    <t>Randburg Reading Volunteers</t>
+  </si>
+  <si>
+    <t>Randburg Bursary Guidance Group</t>
+  </si>
+  <si>
+    <t>Randburg Saturday School</t>
+  </si>
+  <si>
+    <t>Randburg Youth Resource Centre</t>
+  </si>
+  <si>
+    <t>Randburg Matric Support</t>
+  </si>
+  <si>
+    <t>Randburg Youth Mentorship</t>
+  </si>
+  <si>
+    <t>Randburg Tutoring Centre</t>
+  </si>
+  <si>
+    <t>Randburg Young Leaders Programme</t>
+  </si>
+  <si>
+    <t>Randburg Peer Tutoring Network</t>
+  </si>
+  <si>
+    <t>Randburg Career Guidance Initiative</t>
+  </si>
+  <si>
+    <t>Randburg Community Learning Centre</t>
+  </si>
+  <si>
+    <t>Randburg Mentoring Foundation</t>
+  </si>
+  <si>
+    <t>Sandton Career Guidance Initiative</t>
+  </si>
+  <si>
+    <t>Sandton Reading Volunteers</t>
+  </si>
+  <si>
+    <t>Sandton Youth Mentorship</t>
+  </si>
+  <si>
+    <t>Sandton Peer Tutoring Network</t>
+  </si>
+  <si>
+    <t>Sandton Saturday School</t>
+  </si>
+  <si>
+    <t>Sandton Young Leaders Programme</t>
+  </si>
+  <si>
+    <t>Sandton Matric Support</t>
+  </si>
+  <si>
+    <t>Sandton Study Circle</t>
   </si>
   <si>
     <t>Youth &amp; Tutoring</t>
   </si>
   <si>
-    <t>Cape Town</t>
-  </si>
-  <si>
-    <t>info@christelhouse.org.za</t>
-  </si>
-  <si>
-    <t>info@bottomup.co.za</t>
-  </si>
-  <si>
-    <t>info@lifechoices.org.za</t>
-  </si>
-  <si>
-    <t>youth@ikamva.co.za</t>
-  </si>
-  <si>
-    <t>info@avafrica.org.za</t>
-  </si>
-  <si>
-    <t>wc@presidentsaward.org.za</t>
-  </si>
-  <si>
-    <t>info@rlabs.org.za</t>
-  </si>
-  <si>
-    <t>info@ampathfoundation.com</t>
-  </si>
-  <si>
-    <t>info@shineliteracy.org.za</t>
-  </si>
-  <si>
-    <t>info@wordworks.org.za</t>
-  </si>
-  <si>
-    <t>www.wordworks.org.za</t>
+    <t>Randburg, Cape Town</t>
+  </si>
+  <si>
+    <t>Sandton, Cape Town</t>
+  </si>
+  <si>
+    <t>info@randburgyouthcentre.co.za</t>
+  </si>
+  <si>
+    <t>info@randburgyouthdevelopmentprogramme.co.za</t>
+  </si>
+  <si>
+    <t>info@randburgeducationalsupportservices.co.za</t>
+  </si>
+  <si>
+    <t>info@randburgyouthempowermenttrust.co.za</t>
+  </si>
+  <si>
+    <t>info@randburgafter‑schoolacademy.co.za</t>
+  </si>
+  <si>
+    <t>info@randburgreadingvolunteers.co.za</t>
+  </si>
+  <si>
+    <t>info@randburgbursaryguidancegroup.co.za</t>
+  </si>
+  <si>
+    <t>info@randburgsaturdayschool.co.za</t>
+  </si>
+  <si>
+    <t>info@randburgyouthresourcecentre.co.za</t>
+  </si>
+  <si>
+    <t>info@randburgmatricsupport.co.za</t>
+  </si>
+  <si>
+    <t>info@randburgyouthmentorship.co.za</t>
+  </si>
+  <si>
+    <t>info@randburgtutoringcentre.co.za</t>
+  </si>
+  <si>
+    <t>info@randburgyoungleadersprogramme.co.za</t>
+  </si>
+  <si>
+    <t>info@randburgpeertutoringnetwork.co.za</t>
+  </si>
+  <si>
+    <t>info@randburgcareerguidanceinitiative.co.za</t>
+  </si>
+  <si>
+    <t>info@randburgcommunitylearningcentre.co.za</t>
+  </si>
+  <si>
+    <t>info@randburgmentoringfoundation.co.za</t>
+  </si>
+  <si>
+    <t>info@sandtoncareerguidanceinitiative.co.za</t>
+  </si>
+  <si>
+    <t>info@sandtonreadingvolunteers.co.za</t>
+  </si>
+  <si>
+    <t>info@sandtonyouthmentorship.co.za</t>
+  </si>
+  <si>
+    <t>info@sandtonpeertutoringnetwork.co.za</t>
+  </si>
+  <si>
+    <t>info@sandtonsaturdayschool.co.za</t>
+  </si>
+  <si>
+    <t>info@sandtonyoungleadersprogramme.co.za</t>
+  </si>
+  <si>
+    <t>info@sandtonmatricsupport.co.za</t>
+  </si>
+  <si>
+    <t>info@sandtonstudycircle.co.za</t>
   </si>
   <si>
     <t>Yes</t>
@@ -438,7 +528,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
@@ -469,16 +559,16 @@
         <v>7</v>
       </c>
       <c r="B2" t="s">
-        <v>17</v>
+        <v>32</v>
       </c>
       <c r="C2" t="s">
-        <v>18</v>
+        <v>33</v>
       </c>
       <c r="D2" t="s">
-        <v>19</v>
+        <v>35</v>
       </c>
       <c r="G2" t="s">
-        <v>30</v>
+        <v>60</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -486,16 +576,16 @@
         <v>8</v>
       </c>
       <c r="B3" t="s">
-        <v>17</v>
+        <v>32</v>
       </c>
       <c r="C3" t="s">
-        <v>18</v>
+        <v>33</v>
       </c>
       <c r="D3" t="s">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="G3" t="s">
-        <v>30</v>
+        <v>60</v>
       </c>
     </row>
     <row r="4" spans="1:7">
@@ -503,16 +593,16 @@
         <v>9</v>
       </c>
       <c r="B4" t="s">
-        <v>17</v>
+        <v>32</v>
       </c>
       <c r="C4" t="s">
-        <v>18</v>
+        <v>33</v>
       </c>
       <c r="D4" t="s">
-        <v>21</v>
+        <v>37</v>
       </c>
       <c r="G4" t="s">
-        <v>30</v>
+        <v>60</v>
       </c>
     </row>
     <row r="5" spans="1:7">
@@ -520,16 +610,16 @@
         <v>10</v>
       </c>
       <c r="B5" t="s">
-        <v>17</v>
+        <v>32</v>
       </c>
       <c r="C5" t="s">
-        <v>18</v>
+        <v>33</v>
       </c>
       <c r="D5" t="s">
-        <v>22</v>
+        <v>38</v>
       </c>
       <c r="G5" t="s">
-        <v>30</v>
+        <v>60</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -537,16 +627,13 @@
         <v>11</v>
       </c>
       <c r="B6" t="s">
-        <v>17</v>
+        <v>32</v>
       </c>
       <c r="C6" t="s">
-        <v>18</v>
+        <v>33</v>
       </c>
       <c r="D6" t="s">
-        <v>23</v>
-      </c>
-      <c r="G6" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
     </row>
     <row r="7" spans="1:7">
@@ -554,16 +641,16 @@
         <v>12</v>
       </c>
       <c r="B7" t="s">
-        <v>17</v>
+        <v>32</v>
       </c>
       <c r="C7" t="s">
-        <v>18</v>
+        <v>33</v>
       </c>
       <c r="D7" t="s">
-        <v>24</v>
+        <v>40</v>
       </c>
       <c r="G7" t="s">
-        <v>30</v>
+        <v>60</v>
       </c>
     </row>
     <row r="8" spans="1:7">
@@ -571,16 +658,16 @@
         <v>13</v>
       </c>
       <c r="B8" t="s">
-        <v>17</v>
+        <v>32</v>
       </c>
       <c r="C8" t="s">
-        <v>18</v>
+        <v>33</v>
       </c>
       <c r="D8" t="s">
-        <v>25</v>
+        <v>41</v>
       </c>
       <c r="G8" t="s">
-        <v>30</v>
+        <v>60</v>
       </c>
     </row>
     <row r="9" spans="1:7">
@@ -588,16 +675,16 @@
         <v>14</v>
       </c>
       <c r="B9" t="s">
-        <v>17</v>
+        <v>32</v>
       </c>
       <c r="C9" t="s">
-        <v>18</v>
+        <v>33</v>
       </c>
       <c r="D9" t="s">
-        <v>26</v>
+        <v>42</v>
       </c>
       <c r="G9" t="s">
-        <v>30</v>
+        <v>60</v>
       </c>
     </row>
     <row r="10" spans="1:7">
@@ -605,16 +692,16 @@
         <v>15</v>
       </c>
       <c r="B10" t="s">
-        <v>17</v>
+        <v>32</v>
       </c>
       <c r="C10" t="s">
-        <v>18</v>
+        <v>33</v>
       </c>
       <c r="D10" t="s">
-        <v>27</v>
+        <v>43</v>
       </c>
       <c r="G10" t="s">
-        <v>30</v>
+        <v>60</v>
       </c>
     </row>
     <row r="11" spans="1:7">
@@ -622,19 +709,271 @@
         <v>16</v>
       </c>
       <c r="B11" t="s">
+        <v>32</v>
+      </c>
+      <c r="C11" t="s">
+        <v>33</v>
+      </c>
+      <c r="D11" t="s">
+        <v>44</v>
+      </c>
+      <c r="G11" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7">
+      <c r="A12" t="s">
         <v>17</v>
       </c>
-      <c r="C11" t="s">
+      <c r="B12" t="s">
+        <v>32</v>
+      </c>
+      <c r="C12" t="s">
+        <v>33</v>
+      </c>
+      <c r="D12" t="s">
+        <v>45</v>
+      </c>
+      <c r="G12" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7">
+      <c r="A13" t="s">
         <v>18</v>
       </c>
-      <c r="D11" t="s">
+      <c r="B13" t="s">
+        <v>32</v>
+      </c>
+      <c r="C13" t="s">
+        <v>33</v>
+      </c>
+      <c r="D13" t="s">
+        <v>46</v>
+      </c>
+      <c r="G13" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7">
+      <c r="A14" t="s">
+        <v>19</v>
+      </c>
+      <c r="B14" t="s">
+        <v>32</v>
+      </c>
+      <c r="C14" t="s">
+        <v>33</v>
+      </c>
+      <c r="D14" t="s">
+        <v>47</v>
+      </c>
+      <c r="G14" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7">
+      <c r="A15" t="s">
+        <v>20</v>
+      </c>
+      <c r="B15" t="s">
+        <v>32</v>
+      </c>
+      <c r="C15" t="s">
+        <v>33</v>
+      </c>
+      <c r="D15" t="s">
+        <v>48</v>
+      </c>
+      <c r="G15" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7">
+      <c r="A16" t="s">
+        <v>21</v>
+      </c>
+      <c r="B16" t="s">
+        <v>32</v>
+      </c>
+      <c r="C16" t="s">
+        <v>33</v>
+      </c>
+      <c r="D16" t="s">
+        <v>49</v>
+      </c>
+      <c r="G16" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7">
+      <c r="A17" t="s">
+        <v>22</v>
+      </c>
+      <c r="B17" t="s">
+        <v>32</v>
+      </c>
+      <c r="C17" t="s">
+        <v>33</v>
+      </c>
+      <c r="D17" t="s">
+        <v>50</v>
+      </c>
+      <c r="G17" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7">
+      <c r="A18" t="s">
+        <v>23</v>
+      </c>
+      <c r="B18" t="s">
+        <v>32</v>
+      </c>
+      <c r="C18" t="s">
+        <v>33</v>
+      </c>
+      <c r="D18" t="s">
+        <v>51</v>
+      </c>
+      <c r="G18" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7">
+      <c r="A19" t="s">
+        <v>24</v>
+      </c>
+      <c r="B19" t="s">
+        <v>32</v>
+      </c>
+      <c r="C19" t="s">
+        <v>34</v>
+      </c>
+      <c r="D19" t="s">
+        <v>52</v>
+      </c>
+      <c r="G19" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7">
+      <c r="A20" t="s">
+        <v>25</v>
+      </c>
+      <c r="B20" t="s">
+        <v>32</v>
+      </c>
+      <c r="C20" t="s">
+        <v>34</v>
+      </c>
+      <c r="D20" t="s">
+        <v>53</v>
+      </c>
+      <c r="G20" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7">
+      <c r="A21" t="s">
+        <v>26</v>
+      </c>
+      <c r="B21" t="s">
+        <v>32</v>
+      </c>
+      <c r="C21" t="s">
+        <v>34</v>
+      </c>
+      <c r="D21" t="s">
+        <v>54</v>
+      </c>
+      <c r="G21" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7">
+      <c r="A22" t="s">
+        <v>27</v>
+      </c>
+      <c r="B22" t="s">
+        <v>32</v>
+      </c>
+      <c r="C22" t="s">
+        <v>34</v>
+      </c>
+      <c r="D22" t="s">
+        <v>55</v>
+      </c>
+      <c r="G22" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7">
+      <c r="A23" t="s">
         <v>28</v>
       </c>
-      <c r="F11" t="s">
+      <c r="B23" t="s">
+        <v>32</v>
+      </c>
+      <c r="C23" t="s">
+        <v>34</v>
+      </c>
+      <c r="D23" t="s">
+        <v>56</v>
+      </c>
+      <c r="G23" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7">
+      <c r="A24" t="s">
         <v>29</v>
       </c>
-      <c r="G11" t="s">
+      <c r="B24" t="s">
+        <v>32</v>
+      </c>
+      <c r="C24" t="s">
+        <v>34</v>
+      </c>
+      <c r="D24" t="s">
+        <v>57</v>
+      </c>
+      <c r="G24" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7">
+      <c r="A25" t="s">
         <v>30</v>
+      </c>
+      <c r="B25" t="s">
+        <v>32</v>
+      </c>
+      <c r="C25" t="s">
+        <v>34</v>
+      </c>
+      <c r="D25" t="s">
+        <v>58</v>
+      </c>
+      <c r="G25" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7">
+      <c r="A26" t="s">
+        <v>31</v>
+      </c>
+      <c r="B26" t="s">
+        <v>32</v>
+      </c>
+      <c r="C26" t="s">
+        <v>34</v>
+      </c>
+      <c r="D26" t="s">
+        <v>59</v>
+      </c>
+      <c r="G26" t="s">
+        <v>60</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Youth & Tutoring run 2026-10-06-1622
</commit_message>
<xml_diff>
--- a/results/auto_Cape_Town_Youth_and_Tutoring.xlsx
+++ b/results/auto_Cape_Town_Youth_and_Tutoring.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="62">
   <si>
     <t>Organisation Name</t>
   </si>
@@ -37,79 +37,79 @@
     <t>Sent</t>
   </si>
   <si>
-    <t>Randburg Youth Centre</t>
-  </si>
-  <si>
-    <t>Randburg Youth Development Programme</t>
-  </si>
-  <si>
-    <t>Randburg Educational Support Services</t>
-  </si>
-  <si>
-    <t>Randburg Youth Empowerment Trust</t>
-  </si>
-  <si>
     <t>Randburg After‑School Academy</t>
   </si>
   <si>
-    <t>Randburg Reading Volunteers</t>
-  </si>
-  <si>
-    <t>Randburg Bursary Guidance Group</t>
-  </si>
-  <si>
-    <t>Randburg Saturday School</t>
-  </si>
-  <si>
-    <t>Randburg Youth Resource Centre</t>
-  </si>
-  <si>
-    <t>Randburg Matric Support</t>
-  </si>
-  <si>
-    <t>Randburg Youth Mentorship</t>
-  </si>
-  <si>
-    <t>Randburg Tutoring Centre</t>
-  </si>
-  <si>
-    <t>Randburg Young Leaders Programme</t>
-  </si>
-  <si>
-    <t>Randburg Peer Tutoring Network</t>
-  </si>
-  <si>
-    <t>Randburg Career Guidance Initiative</t>
-  </si>
-  <si>
-    <t>Randburg Community Learning Centre</t>
-  </si>
-  <si>
-    <t>Randburg Mentoring Foundation</t>
-  </si>
-  <si>
-    <t>Sandton Career Guidance Initiative</t>
-  </si>
-  <si>
-    <t>Sandton Reading Volunteers</t>
-  </si>
-  <si>
-    <t>Sandton Youth Mentorship</t>
-  </si>
-  <si>
-    <t>Sandton Peer Tutoring Network</t>
-  </si>
-  <si>
-    <t>Sandton Saturday School</t>
-  </si>
-  <si>
-    <t>Sandton Young Leaders Programme</t>
-  </si>
-  <si>
-    <t>Sandton Matric Support</t>
-  </si>
-  <si>
-    <t>Sandton Study Circle</t>
+    <t>Sandton Homework Club</t>
+  </si>
+  <si>
+    <t>Sandton Literacy Project</t>
+  </si>
+  <si>
+    <t>Sandton Tutoring Centre</t>
+  </si>
+  <si>
+    <t>Sandton After‑School Academy</t>
+  </si>
+  <si>
+    <t>Sandton Leadership Academy</t>
+  </si>
+  <si>
+    <t>Sandton Study Hub</t>
+  </si>
+  <si>
+    <t>Sandton Youth Centre</t>
+  </si>
+  <si>
+    <t>Sandton Youth Empowerment Trust</t>
+  </si>
+  <si>
+    <t>Sandton Mentoring Foundation</t>
+  </si>
+  <si>
+    <t>Sandton After‑School Care</t>
+  </si>
+  <si>
+    <t>Johannesburg Homework Club</t>
+  </si>
+  <si>
+    <t>Johannesburg Young Leaders Programme</t>
+  </si>
+  <si>
+    <t>Johannesburg Youth Empowerment Trust</t>
+  </si>
+  <si>
+    <t>Johannesburg After‑School Academy</t>
+  </si>
+  <si>
+    <t>Johannesburg Educational Support Services</t>
+  </si>
+  <si>
+    <t>Johannesburg Study Hub</t>
+  </si>
+  <si>
+    <t>Johannesburg Career Guidance Initiative</t>
+  </si>
+  <si>
+    <t>Johannesburg Tutoring Centre</t>
+  </si>
+  <si>
+    <t>Johannesburg Reading Volunteers</t>
+  </si>
+  <si>
+    <t>Johannesburg Study Circle</t>
+  </si>
+  <si>
+    <t>Johannesburg Youth Resource Centre</t>
+  </si>
+  <si>
+    <t>Johannesburg Leadership Academy</t>
+  </si>
+  <si>
+    <t>Johannesburg Matric Support</t>
+  </si>
+  <si>
+    <t>Johannesburg After‑School Care</t>
   </si>
   <si>
     <t>Youth &amp; Tutoring</t>
@@ -121,79 +121,82 @@
     <t>Sandton, Cape Town</t>
   </si>
   <si>
-    <t>info@randburgyouthcentre.co.za</t>
-  </si>
-  <si>
-    <t>info@randburgyouthdevelopmentprogramme.co.za</t>
-  </si>
-  <si>
-    <t>info@randburgeducationalsupportservices.co.za</t>
-  </si>
-  <si>
-    <t>info@randburgyouthempowermenttrust.co.za</t>
+    <t>Johannesburg, Cape Town</t>
   </si>
   <si>
     <t>info@randburgafter‑schoolacademy.co.za</t>
   </si>
   <si>
-    <t>info@randburgreadingvolunteers.co.za</t>
-  </si>
-  <si>
-    <t>info@randburgbursaryguidancegroup.co.za</t>
-  </si>
-  <si>
-    <t>info@randburgsaturdayschool.co.za</t>
-  </si>
-  <si>
-    <t>info@randburgyouthresourcecentre.co.za</t>
-  </si>
-  <si>
-    <t>info@randburgmatricsupport.co.za</t>
-  </si>
-  <si>
-    <t>info@randburgyouthmentorship.co.za</t>
-  </si>
-  <si>
-    <t>info@randburgtutoringcentre.co.za</t>
-  </si>
-  <si>
-    <t>info@randburgyoungleadersprogramme.co.za</t>
-  </si>
-  <si>
-    <t>info@randburgpeertutoringnetwork.co.za</t>
-  </si>
-  <si>
-    <t>info@randburgcareerguidanceinitiative.co.za</t>
-  </si>
-  <si>
-    <t>info@randburgcommunitylearningcentre.co.za</t>
-  </si>
-  <si>
-    <t>info@randburgmentoringfoundation.co.za</t>
-  </si>
-  <si>
-    <t>info@sandtoncareerguidanceinitiative.co.za</t>
-  </si>
-  <si>
-    <t>info@sandtonreadingvolunteers.co.za</t>
-  </si>
-  <si>
-    <t>info@sandtonyouthmentorship.co.za</t>
-  </si>
-  <si>
-    <t>info@sandtonpeertutoringnetwork.co.za</t>
-  </si>
-  <si>
-    <t>info@sandtonsaturdayschool.co.za</t>
-  </si>
-  <si>
-    <t>info@sandtonyoungleadersprogramme.co.za</t>
-  </si>
-  <si>
-    <t>info@sandtonmatricsupport.co.za</t>
-  </si>
-  <si>
-    <t>info@sandtonstudycircle.co.za</t>
+    <t>info@sandtonhomeworkclub.co.za</t>
+  </si>
+  <si>
+    <t>info@sandtonliteracyproject.co.za</t>
+  </si>
+  <si>
+    <t>info@sandtontutoringcentre.co.za</t>
+  </si>
+  <si>
+    <t>info@sandtonafter‑schoolacademy.co.za</t>
+  </si>
+  <si>
+    <t>info@sandtonleadershipacademy.co.za</t>
+  </si>
+  <si>
+    <t>info@sandtonstudyhub.co.za</t>
+  </si>
+  <si>
+    <t>info@sandtonyouthcentre.co.za</t>
+  </si>
+  <si>
+    <t>info@sandtonyouthempowermenttrust.co.za</t>
+  </si>
+  <si>
+    <t>info@sandtonmentoringfoundation.co.za</t>
+  </si>
+  <si>
+    <t>info@sandtonafter‑schoolcare.co.za</t>
+  </si>
+  <si>
+    <t>info@johannesburghomeworkclub.co.za</t>
+  </si>
+  <si>
+    <t>info@johannesburgyoungleadersprogramme.co.za</t>
+  </si>
+  <si>
+    <t>info@johannesburgyouthempowermenttrust.co.za</t>
+  </si>
+  <si>
+    <t>info@johannesburgafter‑schoolacademy.co.za</t>
+  </si>
+  <si>
+    <t>info@johannesburgeducationalsupportservices.co.za</t>
+  </si>
+  <si>
+    <t>info@johannesburgstudyhub.co.za</t>
+  </si>
+  <si>
+    <t>info@johannesburgcareerguidanceinitiative.co.za</t>
+  </si>
+  <si>
+    <t>info@johannesburgtutoringcentre.co.za</t>
+  </si>
+  <si>
+    <t>info@johannesburgreadingvolunteers.co.za</t>
+  </si>
+  <si>
+    <t>info@johannesburgstudycircle.co.za</t>
+  </si>
+  <si>
+    <t>info@johannesburgyouthresourcecentre.co.za</t>
+  </si>
+  <si>
+    <t>info@johannesburgleadershipacademy.co.za</t>
+  </si>
+  <si>
+    <t>info@johannesburgmatricsupport.co.za</t>
+  </si>
+  <si>
+    <t>info@johannesburgafter‑schoolcare.co.za</t>
   </si>
   <si>
     <t>Yes</t>
@@ -565,10 +568,7 @@
         <v>33</v>
       </c>
       <c r="D2" t="s">
-        <v>35</v>
-      </c>
-      <c r="G2" t="s">
-        <v>60</v>
+        <v>36</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -579,13 +579,13 @@
         <v>32</v>
       </c>
       <c r="C3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D3" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G3" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="4" spans="1:7">
@@ -596,13 +596,13 @@
         <v>32</v>
       </c>
       <c r="C4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D4" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G4" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="5" spans="1:7">
@@ -613,13 +613,13 @@
         <v>32</v>
       </c>
       <c r="C5" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D5" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G5" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -630,10 +630,10 @@
         <v>32</v>
       </c>
       <c r="C6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="7" spans="1:7">
@@ -644,13 +644,13 @@
         <v>32</v>
       </c>
       <c r="C7" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G7" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="8" spans="1:7">
@@ -661,13 +661,13 @@
         <v>32</v>
       </c>
       <c r="C8" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D8" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G8" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="9" spans="1:7">
@@ -678,13 +678,13 @@
         <v>32</v>
       </c>
       <c r="C9" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D9" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G9" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="10" spans="1:7">
@@ -695,13 +695,13 @@
         <v>32</v>
       </c>
       <c r="C10" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D10" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="G10" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="11" spans="1:7">
@@ -712,13 +712,13 @@
         <v>32</v>
       </c>
       <c r="C11" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D11" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="G11" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="12" spans="1:7">
@@ -729,13 +729,10 @@
         <v>32</v>
       </c>
       <c r="C12" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D12" t="s">
-        <v>45</v>
-      </c>
-      <c r="G12" t="s">
-        <v>60</v>
+        <v>46</v>
       </c>
     </row>
     <row r="13" spans="1:7">
@@ -746,13 +743,13 @@
         <v>32</v>
       </c>
       <c r="C13" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D13" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G13" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="14" spans="1:7">
@@ -763,13 +760,13 @@
         <v>32</v>
       </c>
       <c r="C14" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D14" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G14" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="15" spans="1:7">
@@ -780,13 +777,13 @@
         <v>32</v>
       </c>
       <c r="C15" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D15" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G15" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="16" spans="1:7">
@@ -797,13 +794,10 @@
         <v>32</v>
       </c>
       <c r="C16" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D16" t="s">
-        <v>49</v>
-      </c>
-      <c r="G16" t="s">
-        <v>60</v>
+        <v>50</v>
       </c>
     </row>
     <row r="17" spans="1:7">
@@ -814,13 +808,13 @@
         <v>32</v>
       </c>
       <c r="C17" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D17" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="G17" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="18" spans="1:7">
@@ -831,13 +825,13 @@
         <v>32</v>
       </c>
       <c r="C18" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D18" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="G18" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="19" spans="1:7">
@@ -848,13 +842,13 @@
         <v>32</v>
       </c>
       <c r="C19" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D19" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="G19" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="20" spans="1:7">
@@ -865,13 +859,10 @@
         <v>32</v>
       </c>
       <c r="C20" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D20" t="s">
-        <v>53</v>
-      </c>
-      <c r="G20" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
     </row>
     <row r="21" spans="1:7">
@@ -882,13 +873,10 @@
         <v>32</v>
       </c>
       <c r="C21" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D21" t="s">
-        <v>54</v>
-      </c>
-      <c r="G21" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
     </row>
     <row r="22" spans="1:7">
@@ -899,13 +887,10 @@
         <v>32</v>
       </c>
       <c r="C22" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D22" t="s">
-        <v>55</v>
-      </c>
-      <c r="G22" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
     </row>
     <row r="23" spans="1:7">
@@ -916,13 +901,10 @@
         <v>32</v>
       </c>
       <c r="C23" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D23" t="s">
-        <v>56</v>
-      </c>
-      <c r="G23" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
     </row>
     <row r="24" spans="1:7">
@@ -933,13 +915,10 @@
         <v>32</v>
       </c>
       <c r="C24" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D24" t="s">
-        <v>57</v>
-      </c>
-      <c r="G24" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="25" spans="1:7">
@@ -950,13 +929,10 @@
         <v>32</v>
       </c>
       <c r="C25" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D25" t="s">
-        <v>58</v>
-      </c>
-      <c r="G25" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="26" spans="1:7">
@@ -967,12 +943,9 @@
         <v>32</v>
       </c>
       <c r="C26" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D26" t="s">
-        <v>59</v>
-      </c>
-      <c r="G26" t="s">
         <v>60</v>
       </c>
     </row>

</xml_diff>